<commit_message>
docs(entregables): sincronizar vigencia de sesion y estado de TC-46 en capitulo y matriz
</commit_message>
<xml_diff>
--- a/docs/entregables/Matriz_trazabilidad_RF_RNF.xlsx
+++ b/docs/entregables/Matriz_trazabilidad_RF_RNF.xlsx
@@ -1284,7 +1284,7 @@
     <t xml:space="preserve">Se agregó la hoja 'Casos de prueba' con 46 casos ejecutados (45 aprobados y 1 hallazgo de seguridad) y 18 casos pendientes (10 manuales y 8 bloqueados por funcionalidad pendiente). Falta ejecutar los casos con celulares reales y UAT con el cliente, y guardar capturas de la ejecución como evidencia.</t>
   </si>
   <si>
-    <t xml:space="preserve">Ejecutar los casos MAN (celular real y cliente), guardar capturas y, si se acuerda, resolver el hallazgo del token de sesión (TC-46).</t>
+    <t xml:space="preserve">Ejecutar los casos MAN (celular real y cliente), guardar capturas y completar la revocación definitiva del token (TC-46 / Solución B token_version planificada).</t>
   </si>
   <si>
     <t xml:space="preserve">2.1.4.12</t>
@@ -2313,7 +2313,7 @@
     <t xml:space="preserve">Cookie copiada antes del cierre</t>
   </si>
   <si>
-    <t xml:space="preserve">HALLAZGO: la cookie copiada antes del cierre sigue siendo válida hasta que expira (vigencia de 8 h; el token no se revoca en el servidor). RF-03 cumple en el navegador, pero conviene acortar la vigencia o agregar revocación.</t>
+    <t xml:space="preserve">HALLAZGO (Mitigado, no resuelto): la vigencia de sesión se acortó y parametrizó con SESSION_TTL_MINUTES (30 min por defecto, en lugar de 8 h), con manejo de expiración HTTP 401 en frontend. La revocación con token_version quedó planificada como tarea T14.</t>
   </si>
   <si>
     <t xml:space="preserve">MAN-01</t>

</xml_diff>